<commit_message>
Update MIS3371 Contribution Tracker.xlsx
</commit_message>
<xml_diff>
--- a/MIS3371 Contribution Tracker.xlsx
+++ b/MIS3371 Contribution Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uofh-my.sharepoint.com/personal/cnguy231_cougarnet_uh_edu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A17A4CE-04BC-4567-A110-33AB4F329825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{40E8F8A2-DA21-4126-A916-F76A6FD7EBDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="20" windowWidth="23020" windowHeight="14620" xr2:uid="{30688633-D282-4B4F-9CFE-0F6485F2C445}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Team Member</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Sept 16 - Live Build</t>
+  </si>
+  <si>
+    <t>09/21 - Live Build: CSS</t>
+  </si>
+  <si>
+    <t>09/23 - Attendence</t>
   </si>
   <si>
     <t>Lana Tran</t>
@@ -142,7 +148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -180,11 +186,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -214,6 +231,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -550,13 +573,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7064EB42-CD23-49CB-9B54-70C1C4D8618F}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="8" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="78.95" thickBot="1">
+    <row r="1" spans="1:9" ht="78.95" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -578,11 +601,16 @@
       <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5"/>
+      <c r="H1" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="26.45" thickBot="1">
+    <row r="2" spans="1:9" ht="26.45" thickBot="1">
       <c r="A2" s="6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" s="7">
         <v>100</v>
@@ -602,11 +630,16 @@
       <c r="G2" s="8">
         <v>100</v>
       </c>
-      <c r="H2" s="5"/>
+      <c r="H2" s="5">
+        <v>100</v>
+      </c>
+      <c r="I2" s="12">
+        <v>100</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="26.45" thickBot="1">
+    <row r="3" spans="1:9" ht="26.45" thickBot="1">
       <c r="A3" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="7">
         <v>100</v>
@@ -626,11 +659,16 @@
       <c r="G3" s="8">
         <v>100</v>
       </c>
-      <c r="H3" s="5"/>
+      <c r="H3" s="5">
+        <v>100</v>
+      </c>
+      <c r="I3" s="12">
+        <v>100</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" ht="26.45" thickBot="1">
+    <row r="4" spans="1:9" ht="26.45" thickBot="1">
       <c r="A4" s="6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="7">
         <v>100</v>
@@ -650,11 +688,16 @@
       <c r="G4" s="8">
         <v>100</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="5">
+        <v>100</v>
+      </c>
+      <c r="I4" s="12">
+        <v>100</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" ht="26.45" thickBot="1">
+    <row r="5" spans="1:9" ht="26.45" thickBot="1">
       <c r="A5" s="9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="7">
         <v>100</v>
@@ -674,11 +717,16 @@
       <c r="G5" s="8">
         <v>100</v>
       </c>
-      <c r="H5" s="5"/>
+      <c r="H5" s="5">
+        <v>100</v>
+      </c>
+      <c r="I5" s="12">
+        <v>100</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" ht="26.45" thickBot="1">
+    <row r="6" spans="1:9" ht="26.45" thickBot="1">
       <c r="A6" s="6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B6" s="7">
         <v>100</v>
@@ -698,9 +746,14 @@
       <c r="G6" s="8">
         <v>100</v>
       </c>
-      <c r="H6" s="5"/>
+      <c r="H6" s="5">
+        <v>100</v>
+      </c>
+      <c r="I6" s="12">
+        <v>100</v>
+      </c>
     </row>
-    <row r="7" spans="1:8" ht="15" thickBot="1">
+    <row r="7" spans="1:9" ht="15" thickBot="1">
       <c r="A7" s="5"/>
       <c r="B7" s="10"/>
       <c r="C7" s="5"/>
@@ -709,6 +762,7 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -716,23 +770,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="41165478-3f5a-49d8-b2c1-4a6763303165" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D90AFCFB7A108C4F8F8BA976CF505DEC" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cd2c722d48fef0d4ecf736b13d623b42">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="41165478-3f5a-49d8-b2c1-4a6763303165" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b6d5bfc7d9d23387cb55f9b459df9728" ns3:_="">
     <xsd:import namespace="41165478-3f5a-49d8-b2c1-4a6763303165"/>
@@ -882,14 +919,31 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="41165478-3f5a-49d8-b2c1-4a6763303165" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D4D321C-E5D4-40B4-8EE2-EB514AE9DC35}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38074111-C309-4A5A-B2E4-375C5B6267CD}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{793C2600-2A3D-47D3-BF82-7EC71AE0048B}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D4D321C-E5D4-40B4-8EE2-EB514AE9DC35}"/>
 </file>
</xml_diff>

<commit_message>
Revert "Update MIS3371 Contribution Tracker.xlsx"
This reverts commit 6530864351b8f6366c47084d06e12172ba55f595.
</commit_message>
<xml_diff>
--- a/MIS3371 Contribution Tracker.xlsx
+++ b/MIS3371 Contribution Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uofh-my.sharepoint.com/personal/cnguy231_cougarnet_uh_edu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40E8F8A2-DA21-4126-A916-F76A6FD7EBDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A17A4CE-04BC-4567-A110-33AB4F329825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="20" windowWidth="23020" windowHeight="14620" xr2:uid="{30688633-D282-4B4F-9CFE-0F6485F2C445}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Team Member</t>
   </si>
@@ -60,12 +60,6 @@
   </si>
   <si>
     <t>Sept 16 - Live Build</t>
-  </si>
-  <si>
-    <t>09/21 - Live Build: CSS</t>
-  </si>
-  <si>
-    <t>09/23 - Attendence</t>
   </si>
   <si>
     <t>Lana Tran</t>
@@ -148,7 +142,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -186,22 +180,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -231,12 +214,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -573,13 +550,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7064EB42-CD23-49CB-9B54-70C1C4D8618F}">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="7" max="7" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="8" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="78.95" thickBot="1">
+    <row r="1" spans="1:8" ht="78.95" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -601,159 +578,129 @@
       <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="5"/>
+    </row>
+    <row r="2" spans="1:8" ht="26.45" thickBot="1">
+      <c r="A2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="B2" s="7">
+        <v>100</v>
+      </c>
+      <c r="C2" s="7">
+        <v>100</v>
+      </c>
+      <c r="D2" s="7">
+        <v>100</v>
+      </c>
+      <c r="E2" s="7">
+        <v>100</v>
+      </c>
+      <c r="F2" s="7">
+        <v>100</v>
+      </c>
+      <c r="G2" s="8">
+        <v>100</v>
+      </c>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8" ht="26.45" thickBot="1">
+      <c r="A3" s="9" t="s">
         <v>8</v>
       </c>
+      <c r="B3" s="7">
+        <v>100</v>
+      </c>
+      <c r="C3" s="7">
+        <v>100</v>
+      </c>
+      <c r="D3" s="7">
+        <v>100</v>
+      </c>
+      <c r="E3" s="7">
+        <v>100</v>
+      </c>
+      <c r="F3" s="7">
+        <v>100</v>
+      </c>
+      <c r="G3" s="8">
+        <v>100</v>
+      </c>
+      <c r="H3" s="5"/>
     </row>
-    <row r="2" spans="1:9" ht="26.45" thickBot="1">
-      <c r="A2" s="6" t="s">
+    <row r="4" spans="1:8" ht="26.45" thickBot="1">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="7">
-        <v>100</v>
-      </c>
-      <c r="C2" s="7">
-        <v>100</v>
-      </c>
-      <c r="D2" s="7">
-        <v>100</v>
-      </c>
-      <c r="E2" s="7">
-        <v>100</v>
-      </c>
-      <c r="F2" s="7">
-        <v>100</v>
-      </c>
-      <c r="G2" s="8">
-        <v>100</v>
-      </c>
-      <c r="H2" s="5">
-        <v>100</v>
-      </c>
-      <c r="I2" s="12">
-        <v>100</v>
-      </c>
+      <c r="B4" s="7">
+        <v>100</v>
+      </c>
+      <c r="C4" s="7">
+        <v>100</v>
+      </c>
+      <c r="D4" s="7">
+        <v>100</v>
+      </c>
+      <c r="E4" s="7">
+        <v>100</v>
+      </c>
+      <c r="F4" s="7">
+        <v>100</v>
+      </c>
+      <c r="G4" s="8">
+        <v>100</v>
+      </c>
+      <c r="H4" s="5"/>
     </row>
-    <row r="3" spans="1:9" ht="26.45" thickBot="1">
-      <c r="A3" s="9" t="s">
+    <row r="5" spans="1:8" ht="26.45" thickBot="1">
+      <c r="A5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="7">
-        <v>100</v>
-      </c>
-      <c r="C3" s="7">
-        <v>100</v>
-      </c>
-      <c r="D3" s="7">
-        <v>100</v>
-      </c>
-      <c r="E3" s="7">
-        <v>100</v>
-      </c>
-      <c r="F3" s="7">
-        <v>100</v>
-      </c>
-      <c r="G3" s="8">
-        <v>100</v>
-      </c>
-      <c r="H3" s="5">
-        <v>100</v>
-      </c>
-      <c r="I3" s="12">
-        <v>100</v>
-      </c>
+      <c r="B5" s="7">
+        <v>100</v>
+      </c>
+      <c r="C5" s="7">
+        <v>100</v>
+      </c>
+      <c r="D5" s="7">
+        <v>100</v>
+      </c>
+      <c r="E5" s="7">
+        <v>100</v>
+      </c>
+      <c r="F5" s="7">
+        <v>100</v>
+      </c>
+      <c r="G5" s="8">
+        <v>100</v>
+      </c>
+      <c r="H5" s="5"/>
     </row>
-    <row r="4" spans="1:9" ht="26.45" thickBot="1">
-      <c r="A4" s="6" t="s">
+    <row r="6" spans="1:8" ht="26.45" thickBot="1">
+      <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="7">
-        <v>100</v>
-      </c>
-      <c r="C4" s="7">
-        <v>100</v>
-      </c>
-      <c r="D4" s="7">
-        <v>100</v>
-      </c>
-      <c r="E4" s="7">
-        <v>100</v>
-      </c>
-      <c r="F4" s="7">
-        <v>100</v>
-      </c>
-      <c r="G4" s="8">
-        <v>100</v>
-      </c>
-      <c r="H4" s="5">
-        <v>100</v>
-      </c>
-      <c r="I4" s="12">
-        <v>100</v>
-      </c>
+      <c r="B6" s="7">
+        <v>100</v>
+      </c>
+      <c r="C6" s="7">
+        <v>100</v>
+      </c>
+      <c r="D6" s="7">
+        <v>100</v>
+      </c>
+      <c r="E6" s="7">
+        <v>100</v>
+      </c>
+      <c r="F6" s="7">
+        <v>100</v>
+      </c>
+      <c r="G6" s="8">
+        <v>100</v>
+      </c>
+      <c r="H6" s="5"/>
     </row>
-    <row r="5" spans="1:9" ht="26.45" thickBot="1">
-      <c r="A5" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="7">
-        <v>100</v>
-      </c>
-      <c r="C5" s="7">
-        <v>100</v>
-      </c>
-      <c r="D5" s="7">
-        <v>100</v>
-      </c>
-      <c r="E5" s="7">
-        <v>100</v>
-      </c>
-      <c r="F5" s="7">
-        <v>100</v>
-      </c>
-      <c r="G5" s="8">
-        <v>100</v>
-      </c>
-      <c r="H5" s="5">
-        <v>100</v>
-      </c>
-      <c r="I5" s="12">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="26.45" thickBot="1">
-      <c r="A6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="7">
-        <v>100</v>
-      </c>
-      <c r="C6" s="7">
-        <v>100</v>
-      </c>
-      <c r="D6" s="7">
-        <v>100</v>
-      </c>
-      <c r="E6" s="7">
-        <v>100</v>
-      </c>
-      <c r="F6" s="7">
-        <v>100</v>
-      </c>
-      <c r="G6" s="8">
-        <v>100</v>
-      </c>
-      <c r="H6" s="5">
-        <v>100</v>
-      </c>
-      <c r="I6" s="12">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="15" thickBot="1">
+    <row r="7" spans="1:8" ht="15" thickBot="1">
       <c r="A7" s="5"/>
       <c r="B7" s="10"/>
       <c r="C7" s="5"/>
@@ -762,7 +709,6 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -770,6 +716,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="41165478-3f5a-49d8-b2c1-4a6763303165" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D90AFCFB7A108C4F8F8BA976CF505DEC" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="cd2c722d48fef0d4ecf736b13d623b42">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="41165478-3f5a-49d8-b2c1-4a6763303165" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b6d5bfc7d9d23387cb55f9b459df9728" ns3:_="">
     <xsd:import namespace="41165478-3f5a-49d8-b2c1-4a6763303165"/>
@@ -919,31 +882,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="41165478-3f5a-49d8-b2c1-4a6763303165" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38074111-C309-4A5A-B2E4-375C5B6267CD}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{793C2600-2A3D-47D3-BF82-7EC71AE0048B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D4D321C-E5D4-40B4-8EE2-EB514AE9DC35}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38074111-C309-4A5A-B2E4-375C5B6267CD}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{793C2600-2A3D-47D3-BF82-7EC71AE0048B}"/>
 </file>
</xml_diff>